<commit_message>
fix: localize Excel training content to Slovak
</commit_message>
<xml_diff>
--- a/solutions/excel-01-basics.xlsx
+++ b/solutions/excel-01-basics.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predaj" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faktúra" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dochádzka" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -18,14 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.00 [$€-sk-SK];[Red](#,##0.00 [$€-sk-SK]);-"/>
-    <numFmt numFmtId="165" formatCode="0.00%;[Red](0.00%);-"/>
-    <numFmt numFmtId="166" formatCode="#,##0;[Red](#,##0);-"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="168" formatCode="dd.mm.yyyy"/>
-    <numFmt numFmtId="169" formatCode="hh:mm"/>
-    <numFmt numFmtId="170" formatCode="[h]:mm"/>
+    <numFmt numFmtId="165" formatCode="#,##0;[Red](#,##0);-"/>
+    <numFmt numFmtId="166" formatCode="0.00%;[Red](0.00%);-"/>
+    <numFmt numFmtId="167" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="168" formatCode="hh:mm"/>
+    <numFmt numFmtId="169" formatCode="[h]:mm"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -83,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -93,13 +92,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -177,7 +181,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblSalesBasics" displayName="tblSalesBasics" ref="A3:H9" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblPredajZaklady" displayName="tblPredajZaklady" ref="A3:H9" headerRowCount="1">
   <autoFilter ref="A3:H9"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Product"/>
@@ -194,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblAttendanceBasics" displayName="tblAttendanceBasics" ref="A3:G7" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblDochadzkaZaklady" displayName="tblDochadzkaZaklady" ref="A3:G7" headerRowCount="1">
   <autoFilter ref="A3:G7"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Date"/>
@@ -525,47 +529,47 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Produkt</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Kategória</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Unit Price</t>
+          <t>Jednotková cena</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Množstvo</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Tržba</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>VAT Rate</t>
+          <t>Sadzba DPH</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>DPH</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Total incl. VAT</t>
+          <t>Spolu s DPH</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Súhrn</t>
         </is>
       </c>
     </row>
@@ -583,14 +587,14 @@
       <c r="C4" s="4" t="n">
         <v>899</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="12" t="n">
         <v>2</v>
       </c>
       <c r="E4" s="4">
         <f>C4*D4</f>
         <v/>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G4" s="4">
@@ -603,7 +607,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Total Revenue</t>
+          <t>Celková tržba</t>
         </is>
       </c>
       <c r="K4" s="4">
@@ -625,14 +629,14 @@
       <c r="C5" s="4" t="n">
         <v>289</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="12" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="4">
         <f>C5*D5</f>
         <v/>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G5" s="4">
@@ -645,7 +649,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Average Revenue</t>
+          <t>Priemerná tržba</t>
         </is>
       </c>
       <c r="K5" s="4">
@@ -656,7 +660,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Klávesnica Wireless</t>
+          <t>Bezdrôtová klávesnica</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -667,14 +671,14 @@
       <c r="C6" s="4" t="n">
         <v>49.9</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="12" t="n">
         <v>12</v>
       </c>
       <c r="E6" s="4">
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G6" s="4">
@@ -687,7 +691,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Minimum Revenue</t>
+          <t>Minimálna tržba</t>
         </is>
       </c>
       <c r="K6" s="4">
@@ -698,7 +702,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>USB-C Dock</t>
+          <t>Dokovacia stanica USB-C</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -709,14 +713,14 @@
       <c r="C7" s="4" t="n">
         <v>129</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="12" t="n">
         <v>7</v>
       </c>
       <c r="E7" s="4">
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G7" s="4">
@@ -729,7 +733,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Maximum Revenue</t>
+          <t>Maximálna tržba</t>
         </is>
       </c>
       <c r="K7" s="4">
@@ -751,14 +755,14 @@
       <c r="C8" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="12" t="n">
         <v>10</v>
       </c>
       <c r="E8" s="4">
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G8" s="4">
@@ -771,10 +775,10 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="K8" s="5">
+          <t>Počet</t>
+        </is>
+      </c>
+      <c r="K8" s="12">
         <f>COUNT(E4:E9)</f>
         <v/>
       </c>
@@ -782,7 +786,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Office Chair</t>
+          <t>Kancelárska stolička</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -793,14 +797,14 @@
       <c r="C9" s="4" t="n">
         <v>329</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="12" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="4">
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="13" t="n">
         <v>0.23</v>
       </c>
       <c r="G9" s="4">
@@ -852,20 +856,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Invoice No.</t>
+          <t>Číslo faktúry</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INV-TRAIN-001</t>
+          <t>FA-TRÉNING-001</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>VAT Rate</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
+          <t>Sadzba DPH</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
         <v>0.23</v>
       </c>
     </row>
@@ -873,37 +877,37 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Kód</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Produkt</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Množstvo</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Unit Price</t>
+          <t>Jednotková cena</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Net</t>
+          <t>Bez DPH</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>DPH</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Gross</t>
+          <t>S DPH</t>
         </is>
       </c>
     </row>
@@ -975,7 +979,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>USB-C Dock</t>
+          <t>Dokovacia stanica USB-C</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1005,7 +1009,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Headset Office</t>
+          <t>Kancelársky headset</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1085,42 +1089,42 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Dátum</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Employee</t>
+          <t>Zamestnanec</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Príchod</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Departure</t>
+          <t>Odchod</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Break (h)</t>
+          <t>Prestávka (h)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Worked time</t>
+          <t>Odpracovaný čas</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Work mode</t>
+          <t>Režim práce</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="14" t="n">
         <v>46266</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1128,27 +1132,27 @@
           <t>Anna Nováková</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="15" t="n">
         <v>0.3347222222222222</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="15" t="n">
         <v>0.6881944444444444</v>
       </c>
       <c r="E4" t="n">
         <v>0.5</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="16">
         <f>(D4-C4)-E4/24</f>
         <v/>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Kancelária</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="14" t="n">
         <v>46266</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -1156,27 +1160,27 @@
           <t>Peter Horváth</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="15" t="n">
         <v>0.325</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="15" t="n">
         <v>0.6736111111111112</v>
       </c>
       <c r="E5" t="n">
         <v>0.5</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="16">
         <f>(D5-C5)-E5/24</f>
         <v/>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Kancelária</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="14" t="n">
         <v>46267</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -1184,27 +1188,27 @@
           <t>Anna Nováková</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="15" t="n">
         <v>0.3326388888888889</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.6868055555555556</v>
       </c>
       <c r="E6" t="n">
         <v>0.5</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="16">
         <f>(D6-C6)-E6/24</f>
         <v/>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Kancelária</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="14" t="n">
         <v>46267</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -1212,22 +1216,22 @@
           <t>Peter Horváth</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="15" t="n">
         <v>0.3402777777777778</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="15" t="n">
         <v>0.6916666666666667</v>
       </c>
       <c r="E7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="16">
         <f>(D7-C7)-E7/24</f>
         <v/>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Na diaľku</t>
         </is>
       </c>
     </row>

</xml_diff>